<commit_message>
feat: rename fab-tab headers — 爆炸半徑 (1:x) / Tenant (with inline options)
D column '每台上限' -> '爆炸半徑 (1:x), EX: 2'; E column '共居' -> 'Tenant (自由=留空/指定群組/獨佔)'. Headers are display-only (importer reads C/D/E by position, format detection unchanged on C4). Updated exporter, both sample generators, README text, and the exporter test. v2_sample_solver.xlsx not regenerated (open in Excel/locked).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/v2_sample_new_format.xlsx
+++ b/examples/v2_sample_new_format.xlsx
@@ -449,12 +449,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>每台上限</t>
+          <t>爆炸半徑 (1:x), EX: 2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>共居</t>
+          <t>Tenant (自由=留空/指定群組/獨佔)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -608,12 +608,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>每台上限</t>
+          <t>爆炸半徑 (1:x), EX: 2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>共居</t>
+          <t>Tenant (自由=留空/指定群組/獨佔)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>